<commit_message>
fix: rename entity file and add update fields in task spreadsheet
</commit_message>
<xml_diff>
--- a/test_files/csv_test_files/COS10001-Tasks.xlsx
+++ b/test_files/csv_test_files/COS10001-Tasks.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -79,13 +79,16 @@
     <t xml:space="preserve">tutorial_stream</t>
   </si>
   <si>
-    <t xml:space="preserve">has_enabled_numbas_test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">has_numbas_time_delay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">numbas_attempt_limit</t>
+    <t xml:space="preserve">scorm_enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scorm_time_delay_enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scorm_attempt_limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scorm_allow_review</t>
   </si>
   <si>
     <t xml:space="preserve">New Task Def 1</t>
@@ -183,12 +186,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -381,136 +392,139 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr defaultColWidth="10.62109375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="20.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="32.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="24.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="22.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="20.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="32.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="24.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="22.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="0" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="0" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="0" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="0" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="0" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="0" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="0" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="C2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="1" t="b">
+      <c r="F2" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="1" t="b">
+      <c r="H2" s="3" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="I2" s="0" t="n">
+      <c r="I2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="J2" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" s="0" t="s">
+      <c r="J2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="0" t="n">
+      <c r="L2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2" s="1" t="n">
         <v>-1</v>
       </c>
-      <c r="N2" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="O2" s="0" t="n">
+      <c r="N2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="P2" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q2" s="0" t="n">
+      <c r="P2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="R2" s="0" t="s">
-        <v>28</v>
+      <c r="R2" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: add assess in portfolio header to csv tasks test files
</commit_message>
<xml_diff>
--- a/test_files/csv_test_files/COS10001-Tasks.xlsx
+++ b/test_files/csv_test_files/COS10001-Tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aki/dev/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eliya/Dev/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340C3520-A115-9F4A-9A20-57F2A142F36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998BB3C4-F53B-0C49-982F-4CDD259C3970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COS10001-Tasks" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>name</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t>scorm_bypass_test</t>
+  </si>
+  <si>
+    <t>assess_in_portfolio_only</t>
   </si>
 </sst>
 </file>
@@ -359,7 +362,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="19" max="19" width="20.5" customWidth="1"/>
@@ -368,9 +371,10 @@
     <col min="22" max="22" width="22.6640625" customWidth="1"/>
     <col min="23" max="23" width="18.6640625" customWidth="1"/>
     <col min="24" max="24" width="16.83203125" customWidth="1"/>
+    <col min="25" max="25" width="21.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -443,8 +447,11 @@
       <c r="X1" t="s">
         <v>30</v>
       </c>
+      <c r="Y1" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -497,6 +504,9 @@
       </c>
       <c r="R2" t="s">
         <v>29</v>
+      </c>
+      <c r="Y2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enable import of task prerequisites
</commit_message>
<xml_diff>
--- a/test_files/csv_test_files/COS10001-Tasks.xlsx
+++ b/test_files/csv_test_files/COS10001-Tasks.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eliya/Dev/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998BB3C4-F53B-0C49-982F-4CDD259C3970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E229C7F-1118-4C40-BFBA-43524B6E1FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COS10001-Tasks" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>name</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t>assess_in_portfolio_only</t>
+  </si>
+  <si>
+    <t>task_prerequisites</t>
   </si>
 </sst>
 </file>
@@ -362,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="19" max="19" width="20.5" customWidth="1"/>
@@ -372,9 +375,10 @@
     <col min="23" max="23" width="18.6640625" customWidth="1"/>
     <col min="24" max="24" width="16.83203125" customWidth="1"/>
     <col min="25" max="25" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -450,8 +454,11 @@
       <c r="Y1" t="s">
         <v>31</v>
       </c>
+      <c r="Z1" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
chore: export new task definition fields to csv (#523)
* chore: export assess in portfolio property to csv

* chore: add assess in portfolio header to csv tasks test files

* chore: add assess in portfolio header to csv tasks test files

* feat: enable import of task prerequisites

* chore: add task prerequisites header

* test: ensure task prerequisites present in csv

* chore: remove comment

* test: fix task prerequisite csv test
</commit_message>
<xml_diff>
--- a/test_files/csv_test_files/COS10001-Tasks.xlsx
+++ b/test_files/csv_test_files/COS10001-Tasks.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aki/dev/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eliya/Dev/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340C3520-A115-9F4A-9A20-57F2A142F36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E229C7F-1118-4C40-BFBA-43524B6E1FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COS10001-Tasks" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>name</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>scorm_bypass_test</t>
+  </si>
+  <si>
+    <t>assess_in_portfolio_only</t>
+  </si>
+  <si>
+    <t>task_prerequisites</t>
   </si>
 </sst>
 </file>
@@ -359,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="19" max="19" width="20.5" customWidth="1"/>
@@ -368,9 +374,11 @@
     <col min="22" max="22" width="22.6640625" customWidth="1"/>
     <col min="23" max="23" width="18.6640625" customWidth="1"/>
     <col min="24" max="24" width="16.83203125" customWidth="1"/>
+    <col min="25" max="25" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -443,8 +451,14 @@
       <c r="X1" t="s">
         <v>30</v>
       </c>
+      <c r="Y1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -497,6 +511,9 @@
       </c>
       <c r="R2" t="s">
         <v>29</v>
+      </c>
+      <c r="Y2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: add discussion prompts header
</commit_message>
<xml_diff>
--- a/test_files/csv_test_files/COS10001-Tasks.xlsx
+++ b/test_files/csv_test_files/COS10001-Tasks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eliya/Dev/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E229C7F-1118-4C40-BFBA-43524B6E1FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849C7394-8847-1543-B8D9-CBCAA2832C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>name</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>task_prerequisites</t>
+  </si>
+  <si>
+    <t>discussion_prompts</t>
   </si>
 </sst>
 </file>
@@ -365,7 +368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AA2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="19" max="19" width="20.5" customWidth="1"/>
@@ -378,7 +381,7 @@
     <col min="26" max="26" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -457,8 +460,11 @@
       <c r="Z1" t="s">
         <v>32</v>
       </c>
+      <c r="AA1" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
feat: discussion prompts (#546)
* feat: init discussion prompts

* chore: allow created by user to be null

* chore: mount discussion prompt api

* feat: discussion prompt api

* test: ensure discussion prompt permissions

* refactor: check permissions first

* chore: return new entity

* chore: remove unneeded fields

* feat: expose count of discussion prompts

* refactor: simplify discussion prompt schema

* feat: import and export discussion prompts via task definition csv

* test: add discussion prompts header to csv

* chore: rollover discussion prompts

* test: ensure rollover duplicates discussion prompts

* chore: add discussion prompts header

* chore: add discussion prompts header

* test: ensure dicussion prompts are exported to csv

* refactor: remove project specific prompts for task definition

* refactor: remove project specific tests

* chore: add discussion prompts header
</commit_message>
<xml_diff>
--- a/test_files/csv_test_files/COS10001-Tasks.xlsx
+++ b/test_files/csv_test_files/COS10001-Tasks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eliya/Dev/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E229C7F-1118-4C40-BFBA-43524B6E1FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849C7394-8847-1543-B8D9-CBCAA2832C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>name</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>task_prerequisites</t>
+  </si>
+  <si>
+    <t>discussion_prompts</t>
   </si>
 </sst>
 </file>
@@ -365,7 +368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AA2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="19" max="19" width="20.5" customWidth="1"/>
@@ -378,7 +381,7 @@
     <col min="26" max="26" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -457,8 +460,11 @@
       <c r="Z1" t="s">
         <v>32</v>
       </c>
+      <c r="AA1" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>23</v>
       </c>

</xml_diff>